<commit_message>
Ahora si, subiendo el archivo Excel real cerrado
</commit_message>
<xml_diff>
--- a/data/Posiciones.xlsx
+++ b/data/Posiciones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\ADARVE JUV D.H\App_Rendimiento_Futbol\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6948DFCD-A4B4-4D61-9D68-B3A980A8E3F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AAD35BC-AD02-4E4B-8519-96AFC8F921F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4080" yWindow="3720" windowWidth="17280" windowHeight="9960" xr2:uid="{B961EC1D-9D64-4A12-AB9D-930ACB18AE51}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B961EC1D-9D64-4A12-AB9D-930ACB18AE51}"/>
   </bookViews>
   <sheets>
     <sheet name="Posiciones" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="49">
   <si>
     <t>Jugador</t>
   </si>
@@ -164,6 +164,9 @@
   </si>
   <si>
     <t>hasta vuelta sustacha</t>
+  </si>
+  <si>
+    <t>Alex_Palacios</t>
   </si>
 </sst>
 </file>
@@ -708,8 +711,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{97812EF7-7207-445A-B780-D6046FF4E4C8}" name="Tabla1" displayName="Tabla1" ref="A1:D31" totalsRowShown="0">
-  <autoFilter ref="A1:D31" xr:uid="{97812EF7-7207-445A-B780-D6046FF4E4C8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{97812EF7-7207-445A-B780-D6046FF4E4C8}" name="Tabla1" displayName="Tabla1" ref="A1:D32" totalsRowShown="0">
+  <autoFilter ref="A1:D32" xr:uid="{97812EF7-7207-445A-B780-D6046FF4E4C8}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{9890C0E8-1734-48AB-B9B8-F71F9B0FD391}" name="Jugador"/>
     <tableColumn id="2" xr3:uid="{F74319A2-3299-4382-8CC7-D4EC8D8793AD}" name="Posicion"/>
@@ -1017,7 +1020,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86862050-FDEA-4FB1-B5DB-6F278968DFB2}">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.5546875" bestFit="1" customWidth="1"/>
@@ -1460,6 +1463,20 @@
         <v>46</v>
       </c>
     </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>48</v>
+      </c>
+      <c r="B32" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32" t="s">
+        <v>42</v>
+      </c>
+      <c r="D32" t="s">
+        <v>45</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>